<commit_message>
feat: add react export workflows and comps workbook upgrade
Co-Authored-By: Codex CLI
</commit_message>
<xml_diff>
--- a/templates/ticker_review.xlsx
+++ b/templates/ticker_review.xlsx
@@ -15,9 +15,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF_Bull" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equity_Bridge" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QoE" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps Diagnostics" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QoE" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="json_path">Config!$B$2</definedName>
@@ -37,7 +38,7 @@
     <numFmt numFmtId="169" formatCode="+0.0;-0.0;0.0"/>
     <numFmt numFmtId="170" formatCode="+0.0;-0.0"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -159,8 +160,17 @@
       <color rgb="001F3864"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -217,6 +227,24 @@
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F7FA"/>
+        <bgColor rgb="00F5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+        <bgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -241,7 +269,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -513,6 +541,33 @@
     <xf numFmtId="170" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -959,6 +1014,387 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="004F81BD"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="43" t="inlineStr">
+        <is>
+          <t>IBM — SENSITIVITY ANALYSIS  |  IV / Share vs WACC × Terminal Growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  IV/Share ($) — WACC (rows) × Terminal Growth (cols)</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="14" t="n"/>
+      <c r="E2" s="14" t="n"/>
+      <c r="F2" s="14" t="n"/>
+      <c r="G2" s="14" t="n"/>
+      <c r="H2" s="14" t="n"/>
+      <c r="I2" s="14" t="n"/>
+      <c r="J2" s="14" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="82" t="inlineStr">
+        <is>
+          <t>WACC \ Term. g</t>
+        </is>
+      </c>
+      <c r="B3" s="83" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="C3" s="83" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D3" s="83" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="E3" s="83" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F3" s="84" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="G3" s="83" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H3" s="83" t="n">
+        <v>0.04500000000000001</v>
+      </c>
+      <c r="I3" s="83" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J3" s="83" t="n">
+        <v>0.05500000000000001</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="85" t="n">
+        <v>0.05043</v>
+      </c>
+      <c r="B4" s="86" t="n">
+        <v>380.03</v>
+      </c>
+      <c r="C4" s="86" t="n">
+        <v>421.19</v>
+      </c>
+      <c r="D4" s="86" t="n">
+        <v>478.37</v>
+      </c>
+      <c r="E4" s="86" t="n">
+        <v>563.34</v>
+      </c>
+      <c r="F4" s="86" t="n">
+        <v>703.1</v>
+      </c>
+      <c r="G4" s="86" t="n">
+        <v>976.46</v>
+      </c>
+      <c r="H4" s="86" t="n">
+        <v>1752.47</v>
+      </c>
+      <c r="I4" s="86" t="n">
+        <v>20565.41</v>
+      </c>
+      <c r="J4" s="87" t="n">
+        <v>55.18</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="85" t="n">
+        <v>0.05543000000000001</v>
+      </c>
+      <c r="B5" s="86" t="n">
+        <v>323.99</v>
+      </c>
+      <c r="C5" s="86" t="n">
+        <v>352.3</v>
+      </c>
+      <c r="D5" s="86" t="n">
+        <v>389.78</v>
+      </c>
+      <c r="E5" s="86" t="n">
+        <v>441.83</v>
+      </c>
+      <c r="F5" s="86" t="n">
+        <v>519.1799999999999</v>
+      </c>
+      <c r="G5" s="86" t="n">
+        <v>646.38</v>
+      </c>
+      <c r="H5" s="86" t="n">
+        <v>895.17</v>
+      </c>
+      <c r="I5" s="86" t="n">
+        <v>1601.39</v>
+      </c>
+      <c r="J5" s="86" t="n">
+        <v>18722.08</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="85" t="n">
+        <v>0.06043</v>
+      </c>
+      <c r="B6" s="88" t="n">
+        <v>280.4</v>
+      </c>
+      <c r="C6" s="88" t="n">
+        <v>300.54</v>
+      </c>
+      <c r="D6" s="86" t="n">
+        <v>326.25</v>
+      </c>
+      <c r="E6" s="86" t="n">
+        <v>360.29</v>
+      </c>
+      <c r="F6" s="86" t="n">
+        <v>407.56</v>
+      </c>
+      <c r="G6" s="86" t="n">
+        <v>477.78</v>
+      </c>
+      <c r="H6" s="86" t="n">
+        <v>593.26</v>
+      </c>
+      <c r="I6" s="86" t="n">
+        <v>819.1</v>
+      </c>
+      <c r="J6" s="86" t="n">
+        <v>1460.15</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="85" t="n">
+        <v>0.06543</v>
+      </c>
+      <c r="B7" s="88" t="n">
+        <v>245.55</v>
+      </c>
+      <c r="C7" s="88" t="n">
+        <v>260.25</v>
+      </c>
+      <c r="D7" s="88" t="n">
+        <v>278.5</v>
+      </c>
+      <c r="E7" s="88" t="n">
+        <v>301.78</v>
+      </c>
+      <c r="F7" s="86" t="n">
+        <v>332.61</v>
+      </c>
+      <c r="G7" s="86" t="n">
+        <v>375.41</v>
+      </c>
+      <c r="H7" s="86" t="n">
+        <v>438.98</v>
+      </c>
+      <c r="I7" s="86" t="n">
+        <v>543.52</v>
+      </c>
+      <c r="J7" s="86" t="n">
+        <v>747.9299999999999</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="84" t="n">
+        <v>0.07043000000000001</v>
+      </c>
+      <c r="B8" s="87" t="n">
+        <v>217.08</v>
+      </c>
+      <c r="C8" s="87" t="n">
+        <v>228.02</v>
+      </c>
+      <c r="D8" s="88" t="n">
+        <v>241.3</v>
+      </c>
+      <c r="E8" s="88" t="n">
+        <v>257.78</v>
+      </c>
+      <c r="F8" s="89" t="n">
+        <v>278.8</v>
+      </c>
+      <c r="G8" s="86" t="n">
+        <v>306.63</v>
+      </c>
+      <c r="H8" s="86" t="n">
+        <v>345.25</v>
+      </c>
+      <c r="I8" s="86" t="n">
+        <v>402.62</v>
+      </c>
+      <c r="J8" s="86" t="n">
+        <v>496.93</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="85" t="n">
+        <v>0.07543000000000001</v>
+      </c>
+      <c r="B9" s="87" t="n">
+        <v>193.39</v>
+      </c>
+      <c r="C9" s="87" t="n">
+        <v>201.67</v>
+      </c>
+      <c r="D9" s="87" t="n">
+        <v>211.52</v>
+      </c>
+      <c r="E9" s="87" t="n">
+        <v>223.48</v>
+      </c>
+      <c r="F9" s="87" t="n">
+        <v>238.3</v>
+      </c>
+      <c r="G9" s="88" t="n">
+        <v>257.22</v>
+      </c>
+      <c r="H9" s="88" t="n">
+        <v>282.24</v>
+      </c>
+      <c r="I9" s="86" t="n">
+        <v>316.97</v>
+      </c>
+      <c r="J9" s="86" t="n">
+        <v>368.54</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="85" t="n">
+        <v>0.08043</v>
+      </c>
+      <c r="B10" s="87" t="n">
+        <v>173.39</v>
+      </c>
+      <c r="C10" s="87" t="n">
+        <v>179.73</v>
+      </c>
+      <c r="D10" s="87" t="n">
+        <v>187.16</v>
+      </c>
+      <c r="E10" s="87" t="n">
+        <v>196</v>
+      </c>
+      <c r="F10" s="87" t="n">
+        <v>206.71</v>
+      </c>
+      <c r="G10" s="87" t="n">
+        <v>220</v>
+      </c>
+      <c r="H10" s="87" t="n">
+        <v>236.94</v>
+      </c>
+      <c r="I10" s="88" t="n">
+        <v>259.35</v>
+      </c>
+      <c r="J10" s="88" t="n">
+        <v>290.45</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="85" t="n">
+        <v>0.08543000000000001</v>
+      </c>
+      <c r="B11" s="87" t="n">
+        <v>156.29</v>
+      </c>
+      <c r="C11" s="87" t="n">
+        <v>161.19</v>
+      </c>
+      <c r="D11" s="87" t="n">
+        <v>166.86</v>
+      </c>
+      <c r="E11" s="87" t="n">
+        <v>173.49</v>
+      </c>
+      <c r="F11" s="87" t="n">
+        <v>181.38</v>
+      </c>
+      <c r="G11" s="87" t="n">
+        <v>190.94</v>
+      </c>
+      <c r="H11" s="87" t="n">
+        <v>202.79</v>
+      </c>
+      <c r="I11" s="87" t="n">
+        <v>217.9</v>
+      </c>
+      <c r="J11" s="87" t="n">
+        <v>237.88</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="85" t="n">
+        <v>0.09043000000000001</v>
+      </c>
+      <c r="B12" s="87" t="n">
+        <v>141.51</v>
+      </c>
+      <c r="C12" s="87" t="n">
+        <v>145.33</v>
+      </c>
+      <c r="D12" s="87" t="n">
+        <v>149.69</v>
+      </c>
+      <c r="E12" s="87" t="n">
+        <v>154.73</v>
+      </c>
+      <c r="F12" s="87" t="n">
+        <v>160.63</v>
+      </c>
+      <c r="G12" s="87" t="n">
+        <v>167.63</v>
+      </c>
+      <c r="H12" s="87" t="n">
+        <v>176.11</v>
+      </c>
+      <c r="I12" s="87" t="n">
+        <v>186.62</v>
+      </c>
+      <c r="J12" s="87" t="n">
+        <v>200.02</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="90" t="inlineStr">
+        <is>
+          <t>Price = $253.33  |  Green = IV &gt; Price+20%  |  Yellow = within 5%  |  Red = IV &lt; Price-5%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00FFC000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -1243,7 +1679,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001F3864"/>
@@ -1716,7 +2152,7 @@
       </c>
     </row>
     <row r="14" ht="14" customHeight="1">
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="59" t="inlineStr">
         <is>
           <t>Sheet Guide</t>
         </is>
@@ -8030,581 +8466,668 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="58" t="inlineStr">
-        <is>
-          <t>IBM — COMPARABLE COMPANY ANALYSIS</t>
-        </is>
-      </c>
+      <c r="A1" s="103" t="inlineStr">
+        <is>
+          <t>IBM - Comparable Companies Appendix</t>
+        </is>
+      </c>
+      <c r="I1" s="104" t="n"/>
+      <c r="J1" s="104" t="n"/>
+      <c r="K1" s="104" t="n"/>
+      <c r="L1" s="104" t="n"/>
+      <c r="M1" s="104" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
-        <is>
-          <t>Excl.</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="A2" s="105" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B2" s="104" t="inlineStr">
+        <is>
+          <t>International Business Machines</t>
+        </is>
+      </c>
+      <c r="C2" s="104" t="n"/>
+      <c r="D2" s="105" t="inlineStr">
+        <is>
+          <t>As Of</t>
+        </is>
+      </c>
+      <c r="E2" s="104" t="inlineStr">
+        <is>
+          <t>Template Example</t>
+        </is>
+      </c>
+      <c r="F2" s="104" t="n"/>
+      <c r="G2" s="104" t="n"/>
+      <c r="H2" s="104" t="n"/>
+      <c r="I2" s="104" t="n"/>
+      <c r="J2" s="104" t="n"/>
+      <c r="K2" s="104" t="n"/>
+      <c r="L2" s="104" t="n"/>
+      <c r="M2" s="104" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="105" t="inlineStr">
+        <is>
+          <t>Source File</t>
+        </is>
+      </c>
+      <c r="B3" s="104" t="inlineStr">
+        <is>
+          <t>staged export payload</t>
+        </is>
+      </c>
+      <c r="C3" s="104" t="n"/>
+      <c r="D3" s="105" t="inlineStr">
+        <is>
+          <t>Current Price</t>
+        </is>
+      </c>
+      <c r="E3" s="104" t="n">
+        <v>253.33</v>
+      </c>
+      <c r="F3" s="104" t="n"/>
+      <c r="G3" s="104" t="n"/>
+      <c r="H3" s="104" t="n"/>
+      <c r="I3" s="104" t="n"/>
+      <c r="J3" s="104" t="n"/>
+      <c r="K3" s="104" t="n"/>
+      <c r="L3" s="104" t="n"/>
+      <c r="M3" s="104" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="106" t="inlineStr">
+        <is>
+          <t>Headline Valuation</t>
+        </is>
+      </c>
+      <c r="B4" s="104" t="n"/>
+      <c r="C4" s="104" t="n"/>
+      <c r="D4" s="104" t="n"/>
+      <c r="E4" s="104" t="n"/>
+      <c r="F4" s="104" t="n"/>
+      <c r="G4" s="104" t="n"/>
+      <c r="H4" s="104" t="n"/>
+      <c r="I4" s="104" t="n"/>
+      <c r="J4" s="104" t="n"/>
+      <c r="K4" s="104" t="n"/>
+      <c r="L4" s="104" t="n"/>
+      <c r="M4" s="104" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="107" t="inlineStr">
+        <is>
+          <t>Primary Metric</t>
+        </is>
+      </c>
+      <c r="B5" s="104" t="inlineStr">
+        <is>
+          <t>tev_ebitda_ltm</t>
+        </is>
+      </c>
+      <c r="C5" s="104" t="n"/>
+      <c r="D5" s="104" t="n"/>
+      <c r="E5" s="104" t="n"/>
+      <c r="F5" s="104" t="n"/>
+      <c r="G5" s="104" t="n"/>
+      <c r="H5" s="104" t="n"/>
+      <c r="I5" s="104" t="n"/>
+      <c r="J5" s="104" t="n"/>
+      <c r="K5" s="104" t="n"/>
+      <c r="L5" s="104" t="n"/>
+      <c r="M5" s="104" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="107" t="inlineStr">
+        <is>
+          <t>Blended Base IV</t>
+        </is>
+      </c>
+      <c r="B6" s="104" t="n">
+        <v>248</v>
+      </c>
+      <c r="C6" s="104" t="n"/>
+      <c r="D6" s="104" t="n"/>
+      <c r="E6" s="104" t="n"/>
+      <c r="F6" s="104" t="n"/>
+      <c r="G6" s="104" t="n"/>
+      <c r="H6" s="104" t="n"/>
+      <c r="I6" s="104" t="n"/>
+      <c r="J6" s="104" t="n"/>
+      <c r="K6" s="104" t="n"/>
+      <c r="L6" s="104" t="n"/>
+      <c r="M6" s="104" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="107" t="inlineStr">
+        <is>
+          <t>Bear / Base / Bull</t>
+        </is>
+      </c>
+      <c r="B7" s="104" t="inlineStr">
+        <is>
+          <t>225.0 / 252.0 / 281.0</t>
+        </is>
+      </c>
+      <c r="C7" s="104" t="n"/>
+      <c r="D7" s="104" t="n"/>
+      <c r="E7" s="104" t="n"/>
+      <c r="F7" s="104" t="n"/>
+      <c r="G7" s="104" t="n"/>
+      <c r="H7" s="104" t="n"/>
+      <c r="I7" s="104" t="n"/>
+      <c r="J7" s="104" t="n"/>
+      <c r="K7" s="104" t="n"/>
+      <c r="L7" s="104" t="n"/>
+      <c r="M7" s="104" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="107" t="inlineStr">
+        <is>
+          <t>Peer Counts (raw / clean)</t>
+        </is>
+      </c>
+      <c r="B8" s="104" t="inlineStr">
+        <is>
+          <t>8 / 7</t>
+        </is>
+      </c>
+      <c r="C8" s="104" t="n"/>
+      <c r="D8" s="104" t="n"/>
+      <c r="E8" s="104" t="n"/>
+      <c r="F8" s="104" t="n"/>
+      <c r="G8" s="104" t="n"/>
+      <c r="H8" s="104" t="n"/>
+      <c r="I8" s="104" t="n"/>
+      <c r="J8" s="104" t="n"/>
+      <c r="K8" s="104" t="n"/>
+      <c r="L8" s="104" t="n"/>
+      <c r="M8" s="104" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="107" t="inlineStr">
+        <is>
+          <t>Similarity Method</t>
+        </is>
+      </c>
+      <c r="B9" s="104" t="inlineStr">
+        <is>
+          <t>embedding_cosine</t>
+        </is>
+      </c>
+      <c r="C9" s="104" t="n"/>
+      <c r="D9" s="104" t="n"/>
+      <c r="E9" s="104" t="n"/>
+      <c r="F9" s="104" t="n"/>
+      <c r="G9" s="104" t="n"/>
+      <c r="H9" s="104" t="n"/>
+      <c r="I9" s="104" t="n"/>
+      <c r="J9" s="104" t="n"/>
+      <c r="K9" s="104" t="n"/>
+      <c r="L9" s="104" t="n"/>
+      <c r="M9" s="104" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="107" t="inlineStr">
+        <is>
+          <t>Weighting Formula</t>
+        </is>
+      </c>
+      <c r="B10" s="104" t="inlineStr">
+        <is>
+          <t>0.60*description_similarity + 0.40*market_cap_proximity</t>
+        </is>
+      </c>
+      <c r="C10" s="104" t="n"/>
+      <c r="D10" s="104" t="n"/>
+      <c r="E10" s="104" t="n"/>
+      <c r="F10" s="104" t="n"/>
+      <c r="G10" s="104" t="n"/>
+      <c r="H10" s="104" t="n"/>
+      <c r="I10" s="104" t="n"/>
+      <c r="J10" s="104" t="n"/>
+      <c r="K10" s="104" t="n"/>
+      <c r="L10" s="104" t="n"/>
+      <c r="M10" s="104" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="104" t="n"/>
+      <c r="B11" s="104" t="n"/>
+      <c r="C11" s="104" t="n"/>
+      <c r="D11" s="104" t="n"/>
+      <c r="E11" s="104" t="n"/>
+      <c r="F11" s="104" t="n"/>
+      <c r="G11" s="104" t="n"/>
+      <c r="H11" s="104" t="n"/>
+      <c r="I11" s="104" t="n"/>
+      <c r="J11" s="104" t="n"/>
+      <c r="K11" s="104" t="n"/>
+      <c r="L11" s="104" t="n"/>
+      <c r="M11" s="104" t="n"/>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="106" t="inlineStr">
+        <is>
+          <t>Valuation By Metric</t>
+        </is>
+      </c>
+      <c r="B12" s="104" t="n"/>
+      <c r="C12" s="104" t="n"/>
+      <c r="D12" s="104" t="n"/>
+      <c r="E12" s="104" t="n"/>
+      <c r="F12" s="104" t="n"/>
+      <c r="G12" s="104" t="n"/>
+      <c r="H12" s="104" t="n"/>
+      <c r="I12" s="104" t="n"/>
+      <c r="J12" s="104" t="n"/>
+      <c r="K12" s="104" t="n"/>
+      <c r="L12" s="104" t="n"/>
+      <c r="M12" s="104" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="108" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B13" s="108" t="inlineStr">
+        <is>
+          <t>Target Multiple</t>
+        </is>
+      </c>
+      <c r="C13" s="108" t="inlineStr">
+        <is>
+          <t>Peer Median</t>
+        </is>
+      </c>
+      <c r="D13" s="108" t="inlineStr">
+        <is>
+          <t>Bear Multiple</t>
+        </is>
+      </c>
+      <c r="E13" s="108" t="inlineStr">
+        <is>
+          <t>Base Multiple</t>
+        </is>
+      </c>
+      <c r="F13" s="108" t="inlineStr">
+        <is>
+          <t>Bull Multiple</t>
+        </is>
+      </c>
+      <c r="G13" s="108" t="inlineStr">
+        <is>
+          <t>Bear IV</t>
+        </is>
+      </c>
+      <c r="H13" s="108" t="inlineStr">
+        <is>
+          <t>Base IV</t>
+        </is>
+      </c>
+      <c r="I13" s="108" t="inlineStr">
+        <is>
+          <t>Bull IV</t>
+        </is>
+      </c>
+      <c r="J13" s="108" t="inlineStr">
+        <is>
+          <t>N Raw</t>
+        </is>
+      </c>
+      <c r="K13" s="108" t="inlineStr">
+        <is>
+          <t>N Clean</t>
+        </is>
+      </c>
+      <c r="L13" s="108" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="M13" s="104" t="n"/>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="109" t="inlineStr">
+        <is>
+          <t>TEV / EBITDA LTM</t>
+        </is>
+      </c>
+      <c r="B14" s="109" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="C14" s="109" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="D14" s="109" t="n">
+        <v>12</v>
+      </c>
+      <c r="E14" s="109" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="F14" s="109" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="G14" s="109" t="n">
+        <v>225</v>
+      </c>
+      <c r="H14" s="109" t="n">
+        <v>252</v>
+      </c>
+      <c r="I14" s="109" t="n">
+        <v>281</v>
+      </c>
+      <c r="J14" s="109" t="n">
+        <v>8</v>
+      </c>
+      <c r="K14" s="109" t="n">
+        <v>7</v>
+      </c>
+      <c r="L14" s="109" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M14" s="104" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="109" t="inlineStr">
+        <is>
+          <t>P / E LTM</t>
+        </is>
+      </c>
+      <c r="B15" s="109" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="C15" s="109" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="D15" s="109" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="E15" s="109" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="F15" s="109" t="n">
+        <v>21</v>
+      </c>
+      <c r="G15" s="109" t="n">
+        <v>218</v>
+      </c>
+      <c r="H15" s="109" t="n">
+        <v>241</v>
+      </c>
+      <c r="I15" s="109" t="n">
+        <v>266</v>
+      </c>
+      <c r="J15" s="109" t="n">
+        <v>8</v>
+      </c>
+      <c r="K15" s="109" t="n">
+        <v>8</v>
+      </c>
+      <c r="L15" s="109" t="inlineStr"/>
+      <c r="M15" s="104" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="104" t="n"/>
+      <c r="B16" s="104" t="n"/>
+      <c r="C16" s="104" t="n"/>
+      <c r="D16" s="104" t="n"/>
+      <c r="E16" s="104" t="n"/>
+      <c r="F16" s="104" t="n"/>
+      <c r="G16" s="104" t="n"/>
+      <c r="H16" s="104" t="n"/>
+      <c r="I16" s="104" t="n"/>
+      <c r="J16" s="104" t="n"/>
+      <c r="K16" s="104" t="n"/>
+      <c r="L16" s="104" t="n"/>
+      <c r="M16" s="104" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="106" t="inlineStr">
+        <is>
+          <t>Target Vs Peer Benchmarks</t>
+        </is>
+      </c>
+      <c r="B17" s="104" t="n"/>
+      <c r="C17" s="104" t="n"/>
+      <c r="D17" s="104" t="n"/>
+      <c r="E17" s="104" t="n"/>
+      <c r="F17" s="104" t="n"/>
+      <c r="G17" s="104" t="n"/>
+      <c r="H17" s="104" t="n"/>
+      <c r="I17" s="104" t="n"/>
+      <c r="J17" s="104" t="n"/>
+      <c r="K17" s="104" t="n"/>
+      <c r="L17" s="104" t="n"/>
+      <c r="M17" s="104" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="108" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B18" s="108" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="C18" s="108" t="inlineStr">
+        <is>
+          <t>Peer Median</t>
+        </is>
+      </c>
+      <c r="D18" s="108" t="inlineStr">
+        <is>
+          <t>Delta</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="110" t="inlineStr">
+        <is>
+          <t>TEV / EBITDA LTM</t>
+        </is>
+      </c>
+      <c r="B19" s="110" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="C19" s="110" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="D19" s="110" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="110" t="inlineStr">
+        <is>
+          <t>Revenue Growth</t>
+        </is>
+      </c>
+      <c r="B20" s="110" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C20" s="110" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D20" s="110" t="n">
+        <v>-0.02</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="110" t="inlineStr">
+        <is>
+          <t>EBIT Margin</t>
+        </is>
+      </c>
+      <c r="B21" s="110" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="C21" s="110" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="D21" s="110" t="n">
+        <v>-0.03</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="111" t="inlineStr">
+        <is>
+          <t>Peer Table</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="108" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="C2" s="13" t="inlineStr">
+      <c r="B24" s="108" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="D2" s="13" t="inlineStr">
-        <is>
-          <t>MCap $mm</t>
-        </is>
-      </c>
-      <c r="E2" s="13" t="inlineStr">
-        <is>
-          <t>TEV $mm</t>
-        </is>
-      </c>
-      <c r="F2" s="13" t="inlineStr">
-        <is>
-          <t>Revenue $mm</t>
-        </is>
-      </c>
-      <c r="G2" s="13" t="inlineStr">
-        <is>
-          <t>EBITDA $mm</t>
-        </is>
-      </c>
-      <c r="H2" s="13" t="inlineStr">
-        <is>
-          <t>EBIT $mm</t>
-        </is>
-      </c>
-      <c r="I2" s="13" t="inlineStr">
-        <is>
-          <t>EPS</t>
-        </is>
-      </c>
-      <c r="J2" s="13" t="inlineStr">
-        <is>
-          <t>EV/EBITDA LTM</t>
-        </is>
-      </c>
-      <c r="K2" s="13" t="inlineStr">
-        <is>
-          <t>EV/EBITDA Fwd</t>
-        </is>
-      </c>
-      <c r="L2" s="13" t="inlineStr">
-        <is>
-          <t>EV/EBIT</t>
-        </is>
-      </c>
-      <c r="M2" s="13" t="inlineStr">
-        <is>
-          <t>P/E</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="66" t="inlineStr"/>
-      <c r="B3" s="66" t="inlineStr">
-        <is>
-          <t>IBM</t>
-        </is>
-      </c>
-      <c r="C3" s="67" t="inlineStr">
-        <is>
-          <t>International Business Machines Corporation</t>
-        </is>
-      </c>
-      <c r="D3" s="68" t="n">
-        <v>237632</v>
-      </c>
-      <c r="E3" s="68" t="n">
-        <v>293093</v>
-      </c>
-      <c r="F3" s="68" t="n">
-        <v>66799</v>
-      </c>
-      <c r="G3" s="68" t="n"/>
-      <c r="H3" s="68" t="n"/>
-      <c r="I3" s="68" t="n"/>
-      <c r="J3" s="69" t="n">
-        <v>18.184</v>
-      </c>
-      <c r="K3" s="69" t="n"/>
-      <c r="L3" s="69" t="n"/>
-      <c r="M3" s="69" t="n">
-        <v>22.761005</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="70" t="inlineStr"/>
-      <c r="B4" s="70" t="inlineStr">
+      <c r="C24" s="108" t="inlineStr">
+        <is>
+          <t>Similarity Score</t>
+        </is>
+      </c>
+      <c r="D24" s="108" t="inlineStr">
+        <is>
+          <t>Model Weight</t>
+        </is>
+      </c>
+      <c r="E24" s="108" t="inlineStr">
+        <is>
+          <t>Revenue Growth</t>
+        </is>
+      </c>
+      <c r="F24" s="108" t="inlineStr">
+        <is>
+          <t>EBIT Margin</t>
+        </is>
+      </c>
+      <c r="G24" s="108" t="inlineStr">
+        <is>
+          <t>Net Debt / EBITDA</t>
+        </is>
+      </c>
+      <c r="H24" s="108" t="inlineStr">
+        <is>
+          <t>TEV / EBITDA LTM</t>
+        </is>
+      </c>
+      <c r="I24" s="108" t="inlineStr">
+        <is>
+          <t>TEV / EBIT LTM</t>
+        </is>
+      </c>
+      <c r="J24" s="108" t="inlineStr">
+        <is>
+          <t>P / E LTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="110" t="inlineStr">
+        <is>
+          <t>ACN</t>
+        </is>
+      </c>
+      <c r="B25" s="110" t="inlineStr">
+        <is>
+          <t>Accenture</t>
+        </is>
+      </c>
+      <c r="C25" s="110" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="D25" s="110" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="E25" s="110" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F25" s="110" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G25" s="110" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H25" s="110" t="n">
+        <v>13</v>
+      </c>
+      <c r="I25" s="110" t="n">
+        <v>18</v>
+      </c>
+      <c r="J25" s="110" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="110" t="inlineStr">
         <is>
           <t>ORCL</t>
         </is>
       </c>
-      <c r="C4" s="71" t="inlineStr"/>
-      <c r="D4" s="72" t="n">
-        <v>439620.95936</v>
-      </c>
-      <c r="E4" s="72" t="n">
-        <v>552090.95936</v>
-      </c>
-      <c r="F4" s="72" t="n">
-        <v>61016</v>
-      </c>
-      <c r="G4" s="72" t="n">
-        <v>26266</v>
-      </c>
-      <c r="H4" s="72" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="73" t="n">
-        <v>5.32668</v>
-      </c>
-      <c r="J4" s="74" t="n">
-        <v>19.42683</v>
-      </c>
-      <c r="K4" s="74" t="n">
-        <v>13.8225</v>
-      </c>
-      <c r="L4" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="74" t="n">
-        <v>28.71585</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="75" t="inlineStr"/>
-      <c r="B5" s="75" t="inlineStr">
-        <is>
-          <t>ACN</t>
-        </is>
-      </c>
-      <c r="C5" s="76" t="inlineStr"/>
-      <c r="D5" s="77" t="n">
-        <v>132290.95125</v>
-      </c>
-      <c r="E5" s="77" t="n">
-        <v>131892.41825</v>
-      </c>
-      <c r="F5" s="77" t="n">
-        <v>70725.557</v>
-      </c>
-      <c r="G5" s="77" t="n">
-        <v>12458.011</v>
-      </c>
-      <c r="H5" s="77" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="78" t="n">
-        <v>12.08706</v>
-      </c>
-      <c r="J5" s="79" t="n">
-        <v>9.82953</v>
-      </c>
-      <c r="K5" s="79" t="n">
-        <v>7.7932</v>
-      </c>
-      <c r="L5" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="79" t="n">
-        <v>17.78762</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="70" t="inlineStr"/>
-      <c r="B6" s="70" t="inlineStr">
-        <is>
-          <t>HPE</t>
-        </is>
-      </c>
-      <c r="C6" s="71" t="inlineStr"/>
-      <c r="D6" s="72" t="n">
-        <v>28077.7223372</v>
-      </c>
-      <c r="E6" s="72" t="n">
-        <v>47174.7223372</v>
-      </c>
-      <c r="F6" s="72" t="n">
-        <v>34296</v>
-      </c>
-      <c r="G6" s="72" t="n">
-        <v>4491</v>
-      </c>
-      <c r="H6" s="72" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="73" t="n">
-        <v>-0.04456</v>
-      </c>
-      <c r="J6" s="74" t="n">
-        <v>9.66695</v>
-      </c>
-      <c r="K6" s="74" t="n">
-        <v>7.99156</v>
-      </c>
-      <c r="L6" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="74" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="75" t="inlineStr"/>
-      <c r="B7" s="75" t="inlineStr">
-        <is>
-          <t>CTSH</t>
-        </is>
-      </c>
-      <c r="C7" s="76" t="inlineStr"/>
-      <c r="D7" s="77" t="n">
-        <v>31688.6409192</v>
-      </c>
-      <c r="E7" s="77" t="n">
-        <v>30948.6409192</v>
-      </c>
-      <c r="F7" s="77" t="n">
-        <v>21108</v>
-      </c>
-      <c r="G7" s="77" t="n">
-        <v>3834</v>
-      </c>
-      <c r="H7" s="77" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="78" t="n">
-        <v>4.56</v>
-      </c>
-      <c r="J7" s="79" t="n">
-        <v>7.63034</v>
-      </c>
-      <c r="K7" s="79" t="n">
-        <v>7.42554</v>
-      </c>
-      <c r="L7" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="79" t="n">
-        <v>14.5307</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="70" t="inlineStr"/>
-      <c r="B8" s="70" t="inlineStr">
-        <is>
-          <t>SNX</t>
-        </is>
-      </c>
-      <c r="C8" s="71" t="inlineStr"/>
-      <c r="D8" s="72" t="n">
-        <v>12607.5486043</v>
-      </c>
-      <c r="E8" s="72" t="n">
-        <v>15254.1416043</v>
-      </c>
-      <c r="F8" s="72" t="n">
-        <v>62508.086</v>
-      </c>
-      <c r="G8" s="72" t="n">
-        <v>1836.742</v>
-      </c>
-      <c r="H8" s="72" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="73" t="n">
-        <v>9.95013</v>
-      </c>
-      <c r="J8" s="74" t="n">
-        <v>7.72294</v>
-      </c>
-      <c r="K8" s="74" t="n">
-        <v>7.64777</v>
-      </c>
-      <c r="L8" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="74" t="n">
-        <v>15.71538</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="75" t="inlineStr"/>
-      <c r="B9" s="75" t="inlineStr">
-        <is>
-          <t>MSFT</t>
-        </is>
-      </c>
-      <c r="C9" s="76" t="inlineStr"/>
-      <c r="D9" s="77" t="n">
-        <v>3036785.2685568</v>
-      </c>
-      <c r="E9" s="77" t="n">
-        <v>3070601.2685568</v>
-      </c>
-      <c r="F9" s="77" t="n">
-        <v>305453</v>
-      </c>
-      <c r="G9" s="77" t="n">
-        <v>175259</v>
-      </c>
-      <c r="H9" s="77" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="78" t="n">
-        <v>15.98055</v>
-      </c>
-      <c r="J9" s="79" t="n">
-        <v>16.31624</v>
-      </c>
-      <c r="K9" s="79" t="n">
-        <v>14.35137</v>
-      </c>
-      <c r="L9" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="79" t="n">
-        <v>25.59112</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="70" t="inlineStr"/>
-      <c r="B10" s="70" t="inlineStr">
-        <is>
-          <t>DXC</t>
-        </is>
-      </c>
-      <c r="C10" s="71" t="inlineStr"/>
-      <c r="D10" s="72" t="n">
-        <v>2198.391482</v>
-      </c>
-      <c r="E10" s="72" t="n">
-        <v>5058.391482</v>
-      </c>
-      <c r="F10" s="72" t="n">
-        <v>12683</v>
-      </c>
-      <c r="G10" s="72" t="n">
-        <v>1914</v>
-      </c>
-      <c r="H10" s="72" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="73" t="n">
-        <v>2.3206</v>
-      </c>
-      <c r="J10" s="74" t="n">
-        <v>2.21084</v>
-      </c>
-      <c r="K10" s="74" t="n">
-        <v>2.84159</v>
-      </c>
-      <c r="L10" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="74" t="n">
-        <v>5.58045</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="75" t="inlineStr"/>
-      <c r="B11" s="75" t="inlineStr">
-        <is>
-          <t>HON</t>
-        </is>
-      </c>
-      <c r="C11" s="76" t="inlineStr"/>
-      <c r="D11" s="77" t="n">
-        <v>149568.135453</v>
-      </c>
-      <c r="E11" s="77" t="n">
-        <v>173327.135453</v>
-      </c>
-      <c r="F11" s="77" t="n">
-        <v>37442</v>
-      </c>
-      <c r="G11" s="77" t="n">
-        <v>8468</v>
-      </c>
-      <c r="H11" s="77" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="78" t="n">
-        <v>6.88707</v>
-      </c>
-      <c r="J11" s="79" t="n">
-        <v>19.78846</v>
-      </c>
-      <c r="K11" s="79" t="n">
-        <v>17.30579</v>
-      </c>
-      <c r="L11" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="79" t="n">
-        <v>34.16403</v>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  MEDIAN (excluding "x" peers)</t>
-        </is>
-      </c>
-      <c r="B12" s="51" t="n"/>
-      <c r="C12" s="51" t="n"/>
-      <c r="D12" s="51" t="n"/>
-      <c r="E12" s="51" t="n"/>
-      <c r="F12" s="51" t="n"/>
-      <c r="G12" s="51" t="n"/>
-      <c r="H12" s="51" t="n"/>
-      <c r="I12" s="51" t="n"/>
-      <c r="J12" s="80">
-        <f>IFERROR(MEDIAN(IF(A4:A11&lt;&gt;"x",J4:J11)),MEDIAN(J4:J11))</f>
-        <v/>
-      </c>
-      <c r="K12" s="80">
-        <f>IFERROR(MEDIAN(IF(A4:A11&lt;&gt;"x",K4:K11)),MEDIAN(K4:K11))</f>
-        <v/>
-      </c>
-      <c r="L12" s="80">
-        <f>IFERROR(MEDIAN(IF(A4:A11&lt;&gt;"x",L4:L11)),MEDIAN(L4:L11))</f>
-        <v/>
-      </c>
-      <c r="M12" s="80">
-        <f>IFERROR(MEDIAN(IF(A4:A11&lt;&gt;"x",M4:M11)),MEDIAN(M4:M11))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  IMPLIED INTRINSIC VALUE (Comps)</t>
-        </is>
-      </c>
-      <c r="B14" s="81" t="inlineStr">
-        <is>
-          <t>TEV ($mm)</t>
-        </is>
-      </c>
-      <c r="C14" s="81" t="inlineStr">
-        <is>
-          <t>Equity ($mm)</t>
-        </is>
-      </c>
-      <c r="D14" s="81" t="inlineStr">
-        <is>
-          <t>IV/Share</t>
-        </is>
-      </c>
-      <c r="E14" s="81" t="inlineStr">
-        <is>
-          <t>Upside %</t>
-        </is>
-      </c>
-      <c r="F14" s="14" t="n"/>
-      <c r="G14" s="14" t="n"/>
-      <c r="H14" s="14" t="n"/>
-      <c r="I14" s="14" t="n"/>
-      <c r="J14" s="14" t="n"/>
-      <c r="K14" s="14" t="n"/>
-      <c r="L14" s="14" t="n"/>
-      <c r="M14" s="14" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="17" t="inlineStr">
-        <is>
-          <t>EV/EBITDA LTM approach</t>
-        </is>
-      </c>
-      <c r="B15" s="40">
-        <f>J12*(=Assumptions!$D$3*(Assumptions!$D$8+Assumptions!$D$11))</f>
-        <v/>
-      </c>
-      <c r="C15" s="40">
-        <f>B15+Assumptions!$D$42-(Assumptions!$D$39+Assumptions!$D$43+Assumptions!$D$44+Assumptions!$D$45+Assumptions!$D$46+Assumptions!$D$47+Assumptions!$D$48)</f>
-        <v/>
-      </c>
-      <c r="D15" s="64">
-        <f>C15/Assumptions!$D$40</f>
-        <v/>
-      </c>
-      <c r="E15" s="20">
-        <f>D15/253.33-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>EV/EBIT LTM approach</t>
-        </is>
-      </c>
-      <c r="B16" s="40">
-        <f>L12*Assumptions!$D$3*Assumptions!$D$8</f>
-        <v/>
-      </c>
-      <c r="C16" s="40">
-        <f>B16+Assumptions!$D$42-(Assumptions!$D$39+Assumptions!$D$43+Assumptions!$D$44+Assumptions!$D$45+Assumptions!$D$46+Assumptions!$D$47+Assumptions!$D$48)</f>
-        <v/>
-      </c>
-      <c r="D16" s="64">
-        <f>C16/Assumptions!$D$40</f>
-        <v/>
-      </c>
-      <c r="E16" s="20">
-        <f>D16/253.33-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>P/E approach</t>
-        </is>
-      </c>
-      <c r="B17" s="40">
-        <f>(M12*Assumptions!$D$3*Assumptions!$D$8*(1-Assumptions!$D$14)+Assumptions!$D$42-(Assumptions!$D$39+Assumptions!$D$43+Assumptions!$D$44+Assumptions!$D$45+Assumptions!$D$46+Assumptions!$D$47+Assumptions!$D$48))</f>
-        <v/>
-      </c>
-      <c r="C17" s="40">
-        <f>B17+Assumptions!$D$42-(Assumptions!$D$39+Assumptions!$D$43+Assumptions!$D$44+Assumptions!$D$45+Assumptions!$D$46+Assumptions!$D$47+Assumptions!$D$48)</f>
-        <v/>
-      </c>
-      <c r="D17" s="64">
-        <f>C17/Assumptions!$D$40</f>
-        <v/>
-      </c>
-      <c r="E17" s="20">
-        <f>D17/253.33-1</f>
-        <v/>
+      <c r="B26" s="110" t="inlineStr">
+        <is>
+          <t>Oracle</t>
+        </is>
+      </c>
+      <c r="C26" s="110" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="D26" s="110" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E26" s="110" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="F26" s="110" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G26" s="110" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H26" s="110" t="n">
+        <v>11</v>
+      </c>
+      <c r="I26" s="110" t="n">
+        <v>16</v>
+      </c>
+      <c r="J26" s="110" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8613,379 +9136,336 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="004F81BD"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="43" t="inlineStr">
-        <is>
-          <t>IBM — SENSITIVITY ANALYSIS  |  IV / Share vs WACC × Terminal Growth</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  IV/Share ($) — WACC (rows) × Terminal Growth (cols)</t>
-        </is>
-      </c>
-      <c r="B2" s="14" t="n"/>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="14" t="n"/>
-      <c r="G2" s="14" t="n"/>
-      <c r="H2" s="14" t="n"/>
-      <c r="I2" s="14" t="n"/>
-      <c r="J2" s="14" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="82" t="inlineStr">
-        <is>
-          <t>WACC \ Term. g</t>
-        </is>
-      </c>
-      <c r="B3" s="83" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="C3" s="83" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="D3" s="83" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="E3" s="83" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="F3" s="84" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="G3" s="83" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="H3" s="83" t="n">
-        <v>0.04500000000000001</v>
-      </c>
-      <c r="I3" s="83" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="J3" s="83" t="n">
-        <v>0.05500000000000001</v>
+      <c r="A1" s="112" t="inlineStr">
+        <is>
+          <t>IBM - Comps Diagnostics</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="85" t="n">
-        <v>0.05043</v>
-      </c>
-      <c r="B4" s="86" t="n">
-        <v>380.03</v>
-      </c>
-      <c r="C4" s="86" t="n">
-        <v>421.19</v>
-      </c>
-      <c r="D4" s="86" t="n">
-        <v>478.37</v>
-      </c>
-      <c r="E4" s="86" t="n">
-        <v>563.34</v>
-      </c>
-      <c r="F4" s="86" t="n">
-        <v>703.1</v>
-      </c>
-      <c r="G4" s="86" t="n">
-        <v>976.46</v>
-      </c>
-      <c r="H4" s="86" t="n">
-        <v>1752.47</v>
-      </c>
-      <c r="I4" s="86" t="n">
-        <v>20565.41</v>
-      </c>
-      <c r="J4" s="87" t="n">
-        <v>55.18</v>
+      <c r="A4" s="111" t="inlineStr">
+        <is>
+          <t>Audit Flags</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="85" t="n">
-        <v>0.05543000000000001</v>
-      </c>
-      <c r="B5" s="86" t="n">
-        <v>323.99</v>
-      </c>
-      <c r="C5" s="86" t="n">
-        <v>352.3</v>
-      </c>
-      <c r="D5" s="86" t="n">
-        <v>389.78</v>
-      </c>
-      <c r="E5" s="86" t="n">
-        <v>441.83</v>
-      </c>
-      <c r="F5" s="86" t="n">
-        <v>519.1799999999999</v>
-      </c>
-      <c r="G5" s="86" t="n">
-        <v>646.38</v>
-      </c>
-      <c r="H5" s="86" t="n">
-        <v>895.17</v>
-      </c>
-      <c r="I5" s="86" t="n">
-        <v>1601.39</v>
-      </c>
-      <c r="J5" s="86" t="n">
-        <v>18722.08</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Peer set cleaned from 8 to 7</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="85" t="n">
-        <v>0.06043</v>
-      </c>
-      <c r="B6" s="88" t="n">
-        <v>280.4</v>
-      </c>
-      <c r="C6" s="88" t="n">
-        <v>300.54</v>
-      </c>
-      <c r="D6" s="86" t="n">
-        <v>326.25</v>
-      </c>
-      <c r="E6" s="86" t="n">
-        <v>360.29</v>
-      </c>
-      <c r="F6" s="86" t="n">
-        <v>407.56</v>
-      </c>
-      <c r="G6" s="86" t="n">
-        <v>477.78</v>
-      </c>
-      <c r="H6" s="86" t="n">
-        <v>593.26</v>
-      </c>
-      <c r="I6" s="86" t="n">
-        <v>819.1</v>
-      </c>
-      <c r="J6" s="86" t="n">
-        <v>1460.15</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="85" t="n">
-        <v>0.06543</v>
-      </c>
-      <c r="B7" s="88" t="n">
-        <v>245.55</v>
-      </c>
-      <c r="C7" s="88" t="n">
-        <v>260.25</v>
-      </c>
-      <c r="D7" s="88" t="n">
-        <v>278.5</v>
-      </c>
-      <c r="E7" s="88" t="n">
-        <v>301.78</v>
-      </c>
-      <c r="F7" s="86" t="n">
-        <v>332.61</v>
-      </c>
-      <c r="G7" s="86" t="n">
-        <v>375.41</v>
-      </c>
-      <c r="H7" s="86" t="n">
-        <v>438.98</v>
-      </c>
-      <c r="I7" s="86" t="n">
-        <v>543.52</v>
-      </c>
-      <c r="J7" s="86" t="n">
-        <v>747.9299999999999</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Outliers removed from pe_ltm: ORCL</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="84" t="n">
-        <v>0.07043000000000001</v>
-      </c>
-      <c r="B8" s="87" t="n">
-        <v>217.08</v>
-      </c>
-      <c r="C8" s="87" t="n">
-        <v>228.02</v>
-      </c>
-      <c r="D8" s="88" t="n">
-        <v>241.3</v>
-      </c>
-      <c r="E8" s="88" t="n">
-        <v>257.78</v>
-      </c>
-      <c r="F8" s="89" t="n">
-        <v>278.8</v>
-      </c>
-      <c r="G8" s="86" t="n">
-        <v>306.63</v>
-      </c>
-      <c r="H8" s="86" t="n">
-        <v>345.25</v>
-      </c>
-      <c r="I8" s="86" t="n">
-        <v>402.62</v>
-      </c>
-      <c r="J8" s="86" t="n">
-        <v>496.93</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="85" t="n">
-        <v>0.07543000000000001</v>
-      </c>
-      <c r="B9" s="87" t="n">
-        <v>193.39</v>
-      </c>
-      <c r="C9" s="87" t="n">
-        <v>201.67</v>
-      </c>
-      <c r="D9" s="87" t="n">
-        <v>211.52</v>
-      </c>
-      <c r="E9" s="87" t="n">
-        <v>223.48</v>
-      </c>
-      <c r="F9" s="87" t="n">
-        <v>238.3</v>
-      </c>
-      <c r="G9" s="88" t="n">
-        <v>257.22</v>
-      </c>
-      <c r="H9" s="88" t="n">
-        <v>282.24</v>
-      </c>
-      <c r="I9" s="86" t="n">
-        <v>316.97</v>
-      </c>
-      <c r="J9" s="86" t="n">
-        <v>368.54</v>
+      <c r="A8" s="113" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Template example only; live exports populate from JSON payload.</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="85" t="n">
-        <v>0.08043</v>
-      </c>
-      <c r="B10" s="87" t="n">
-        <v>173.39</v>
-      </c>
-      <c r="C10" s="87" t="n">
-        <v>179.73</v>
-      </c>
-      <c r="D10" s="87" t="n">
-        <v>187.16</v>
-      </c>
-      <c r="E10" s="87" t="n">
-        <v>196</v>
-      </c>
-      <c r="F10" s="87" t="n">
-        <v>206.71</v>
-      </c>
-      <c r="G10" s="87" t="n">
-        <v>220</v>
-      </c>
-      <c r="H10" s="87" t="n">
-        <v>236.94</v>
-      </c>
-      <c r="I10" s="88" t="n">
-        <v>259.35</v>
-      </c>
-      <c r="J10" s="88" t="n">
-        <v>290.45</v>
+      <c r="A10" s="111" t="inlineStr">
+        <is>
+          <t>Metric Status</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="85" t="n">
-        <v>0.08543000000000001</v>
-      </c>
-      <c r="B11" s="87" t="n">
-        <v>156.29</v>
-      </c>
-      <c r="C11" s="87" t="n">
-        <v>161.19</v>
-      </c>
-      <c r="D11" s="87" t="n">
-        <v>166.86</v>
-      </c>
-      <c r="E11" s="87" t="n">
-        <v>173.49</v>
-      </c>
-      <c r="F11" s="87" t="n">
-        <v>181.38</v>
-      </c>
-      <c r="G11" s="87" t="n">
-        <v>190.94</v>
-      </c>
-      <c r="H11" s="87" t="n">
-        <v>202.79</v>
-      </c>
-      <c r="I11" s="87" t="n">
-        <v>217.9</v>
-      </c>
-      <c r="J11" s="87" t="n">
-        <v>237.88</v>
+      <c r="A11" s="108" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B11" s="108" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C11" s="108" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="D11" s="108" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="E11" s="108" t="inlineStr">
+        <is>
+          <t>Raw Multiple</t>
+        </is>
+      </c>
+      <c r="F11" s="108" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="85" t="n">
-        <v>0.09043000000000001</v>
-      </c>
-      <c r="B12" s="87" t="n">
-        <v>141.51</v>
-      </c>
-      <c r="C12" s="87" t="n">
-        <v>145.33</v>
-      </c>
-      <c r="D12" s="87" t="n">
-        <v>149.69</v>
-      </c>
-      <c r="E12" s="87" t="n">
-        <v>154.73</v>
-      </c>
-      <c r="F12" s="87" t="n">
-        <v>160.63</v>
-      </c>
-      <c r="G12" s="87" t="n">
-        <v>167.63</v>
-      </c>
-      <c r="H12" s="87" t="n">
-        <v>176.11</v>
-      </c>
-      <c r="I12" s="87" t="n">
-        <v>186.62</v>
-      </c>
-      <c r="J12" s="87" t="n">
-        <v>200.02</v>
+      <c r="A12" s="110" t="inlineStr">
+        <is>
+          <t>ACN</t>
+        </is>
+      </c>
+      <c r="B12" s="110" t="inlineStr">
+        <is>
+          <t>Accenture</t>
+        </is>
+      </c>
+      <c r="C12" s="110" t="inlineStr">
+        <is>
+          <t>tev_ebitda_ltm</t>
+        </is>
+      </c>
+      <c r="D12" s="110" t="inlineStr">
+        <is>
+          <t>TEV / EBITDA LTM</t>
+        </is>
+      </c>
+      <c r="E12" s="110" t="n">
+        <v>13</v>
+      </c>
+      <c r="F12" s="110" t="inlineStr">
+        <is>
+          <t>included</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="110" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="B13" s="110" t="inlineStr">
+        <is>
+          <t>Oracle</t>
+        </is>
+      </c>
+      <c r="C13" s="110" t="inlineStr">
+        <is>
+          <t>tev_ebitda_ltm</t>
+        </is>
+      </c>
+      <c r="D13" s="110" t="inlineStr">
+        <is>
+          <t>TEV / EBITDA LTM</t>
+        </is>
+      </c>
+      <c r="E13" s="110" t="n">
+        <v>11</v>
+      </c>
+      <c r="F13" s="110" t="inlineStr">
+        <is>
+          <t>included</t>
+        </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="90" t="inlineStr">
-        <is>
-          <t>Price = $253.33  |  Green = IV &gt; Price+20%  |  Yellow = within 5%  |  Red = IV &lt; Price-5%</t>
-        </is>
+      <c r="A14" s="110" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="B14" s="110" t="inlineStr">
+        <is>
+          <t>Oracle</t>
+        </is>
+      </c>
+      <c r="C14" s="110" t="inlineStr">
+        <is>
+          <t>pe_ltm</t>
+        </is>
+      </c>
+      <c r="D14" s="110" t="inlineStr">
+        <is>
+          <t>P / E LTM</t>
+        </is>
+      </c>
+      <c r="E14" s="110" t="n">
+        <v>20</v>
+      </c>
+      <c r="F14" s="110" t="inlineStr">
+        <is>
+          <t>outlier_removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="111" t="inlineStr">
+        <is>
+          <t>Football Field</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="108" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="B17" s="108" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="C17" s="108" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D17" s="108" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="110" t="inlineStr">
+        <is>
+          <t>TEV / EBITDA LTM</t>
+        </is>
+      </c>
+      <c r="B18" s="110" t="n">
+        <v>225</v>
+      </c>
+      <c r="C18" s="110" t="n">
+        <v>252</v>
+      </c>
+      <c r="D18" s="110" t="n">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="110" t="inlineStr">
+        <is>
+          <t>P / E LTM</t>
+        </is>
+      </c>
+      <c r="B19" s="110" t="n">
+        <v>218</v>
+      </c>
+      <c r="C19" s="110" t="n">
+        <v>241</v>
+      </c>
+      <c r="D19" s="110" t="n">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="111" t="inlineStr">
+        <is>
+          <t>Historical Multiples Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="108" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B22" s="108" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C22" s="108" t="inlineStr">
+        <is>
+          <t>Median</t>
+        </is>
+      </c>
+      <c r="D22" s="108" t="inlineStr">
+        <is>
+          <t>P25</t>
+        </is>
+      </c>
+      <c r="E22" s="108" t="inlineStr">
+        <is>
+          <t>P75</t>
+        </is>
+      </c>
+      <c r="F22" s="108" t="inlineStr">
+        <is>
+          <t>Current Percentile</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="110" t="inlineStr">
+        <is>
+          <t>pe_trailing</t>
+        </is>
+      </c>
+      <c r="B23" s="110" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="C23" s="110" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="D23" s="110" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="E23" s="110" t="n">
+        <v>21</v>
+      </c>
+      <c r="F23" s="110" t="n">
+        <v>0.74</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="110" t="inlineStr">
+        <is>
+          <t>ev_ebitda</t>
+        </is>
+      </c>
+      <c r="B24" s="110" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="C24" s="110" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="D24" s="110" t="n">
+        <v>12</v>
+      </c>
+      <c r="E24" s="110" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="F24" s="110" t="n">
+        <v>0.82</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>